<commit_message>
Add value[x] constraint for CodeableConcept (#276) e775a5485eb3b28f95c1a0ec6b3a072fb7ba4497
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-core-organization-type-activite.xlsx
+++ b/main/ig/StructureDefinition-fr-core-organization-type-activite.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="110">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-04T13:09:39+00:00</t>
+    <t>2026-02-09T06:47:58+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -334,44 +334,24 @@
     <t>Extension.value[x]</t>
   </si>
   <si>
-    <t>base64Binary
-booleancanonicalcodedatedateTimedecimalidinstantintegermarkdownoidpositiveIntstringtimeunsignedInturiurluuidAddressAgeAnnotationAttachmentCodeableConceptCodingContactPointCountDistanceDurationHumanNameIdentifierMoneyPeriodQuantityRangeRatioReferenceSampledDataSignatureTimingContactDetailContributorDataRequirementExpressionParameterDefinitionRelatedArtifactTriggerDefinitionUsageContextDosageMeta</t>
-  </si>
-  <si>
-    <t>Value of extension</t>
-  </si>
-  <si>
-    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type:$this}
+    <t xml:space="preserve">CodeableConcept
 </t>
+  </si>
+  <si>
+    <t>Type d'activité</t>
+  </si>
+  <si>
+    <t>Type d'activité de l'UF</t>
+  </si>
+  <si>
+    <t>required</t>
+  </si>
+  <si>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-oragnization-type-activite|2.2.0-ballot-2</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
 </t>
-  </si>
-  <si>
-    <t>Extension.value[x]:valueCodeableConcept</t>
-  </si>
-  <si>
-    <t>valueCodeableConcept</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CodeableConcept
-</t>
-  </si>
-  <si>
-    <t>Type d'activité</t>
-  </si>
-  <si>
-    <t>Type d'activité de l'UF</t>
-  </si>
-  <si>
-    <t>required</t>
-  </si>
-  <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-oragnization-type-activite|2.2.0-ballot-2</t>
   </si>
 </sst>
 </file>
@@ -689,12 +669,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK7"/>
+  <dimension ref="A1:AK6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="34.2734375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="16.80078125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="16.80078125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="19.078125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
@@ -702,7 +682,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="255.0" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="14.78515625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1318,26 +1298,26 @@
         <v>77</v>
       </c>
       <c r="X6" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y6" t="s" s="2">
-        <v>77</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="Y6" s="2"/>
       <c r="Z6" t="s" s="2">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="AA6" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AB6" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AC6" s="2"/>
+        <v>77</v>
+      </c>
+      <c r="AC6" t="s" s="2">
+        <v>77</v>
+      </c>
       <c r="AD6" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE6" t="s" s="2">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="AF6" t="s" s="2">
         <v>103</v>
@@ -1352,112 +1332,9 @@
         <v>77</v>
       </c>
       <c r="AJ6" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AK6" t="s" s="2">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="B7" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="C7" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="D7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E7" s="2"/>
-      <c r="F7" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G7" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K7" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="L7" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="M7" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q7" s="2"/>
-      <c r="R7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X7" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="Y7" s="2"/>
-      <c r="Z7" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="AA7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF7" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AG7" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH7" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI7" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ7" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="AK7" t="s" s="2">
         <v>102</v>
       </c>
     </row>

</xml_diff>